<commit_message>
docs: update Scrum artifacts through HU-029
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Scrum/06_Product_Backlog_CitaJusta.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Scrum/06_Product_Backlog_CitaJusta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC2\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A706AFB5-ECE1-44FC-ADC0-A5F854416DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0283C69-72E1-45CA-82DD-B67C8790A5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="289">
   <si>
     <t>CITAJUSTA  PRODUCT BACKLOG PRIORIZADO</t>
   </si>
@@ -267,6 +267,15 @@
     <t>Sólo se permite una espera activa equivalente cuando así lo defina la regla de negocio. • Se registran servicio, sede/preferencias y fecha de ingreso. • El usuario puede consultar el estado de la espera.</t>
   </si>
   <si>
+    <t>feat/waitlist-entry</t>
+  </si>
+  <si>
+    <t>HU-007 · Done</t>
+  </si>
+  <si>
+    <t>Alta y consulta de lista de espera implementadas y validadas contra PostgreSQL real.</t>
+  </si>
+  <si>
     <t>HU-008</t>
   </si>
   <si>
@@ -282,6 +291,15 @@
     <t>Las preferencias deben usar valores válidos. • Los cambios aplican a futuras evaluaciones de compatibilidad. • El usuario puede retirarse de una espera activa y el cambio queda persistido.</t>
   </si>
   <si>
+    <t>feat/waitlist-preferences</t>
+  </si>
+  <si>
+    <t>HU-008 · Done</t>
+  </si>
+  <si>
+    <t>Preferencias y retiro implementados; E2E HU-007/HU-008 real 24/24 PASS.</t>
+  </si>
+  <si>
     <t>HU-009</t>
   </si>
   <si>
@@ -303,6 +321,15 @@
     <t>La oferta sólo se genera para un candidato compatible. • La oferta posee fecha/hora de expiración persistida. • El usuario es notificado dentro de CitaJusta.</t>
   </si>
   <si>
+    <t>feat/reassignment-offers</t>
+  </si>
+  <si>
+    <t>HU-009 · Done</t>
+  </si>
+  <si>
+    <t>Generación de oferta, ranking/snapshot y TTL implementados en backend.</t>
+  </si>
+  <si>
     <t>HU-010</t>
   </si>
   <si>
@@ -318,6 +345,15 @@
     <t>Sólo el destinatario puede aceptar la oferta. • La oferta debe estar vigente y el cupo disponible. • La aceptación se ejecuta transaccionalmente.</t>
   </si>
   <si>
+    <t>feat/accept-reassignment-offer</t>
+  </si>
+  <si>
+    <t>HU-010 · Done</t>
+  </si>
+  <si>
+    <t>Aceptación transaccional e idempotente implementada con transferencia segura de la cita.</t>
+  </si>
+  <si>
     <t>HU-011</t>
   </si>
   <si>
@@ -333,6 +369,15 @@
     <t>Sólo el destinatario puede rechazar. • La oferta cambia a estado rechazado. • El cupo puede continuar con el siguiente candidato válido.</t>
   </si>
   <si>
+    <t>feat/reject-reassignment-offer</t>
+  </si>
+  <si>
+    <t>HU-011 · Done</t>
+  </si>
+  <si>
+    <t>Rechazo y continuidad/exhaustión del flujo implementados.</t>
+  </si>
+  <si>
     <t>HU-012</t>
   </si>
   <si>
@@ -351,6 +396,15 @@
     <t>Sólo roles autorizados pueden crear o modificar datos institucionales. • Una sede pertenece a una institución válida. • Un servicio puede activarse o desactivarse sin borrar su historial.</t>
   </si>
   <si>
+    <t>feat/catalog-administration</t>
+  </si>
+  <si>
+    <t>HU-012 · Done</t>
+  </si>
+  <si>
+    <t>Administración de sedes/servicios implementada con permisos y activación/desactivación.</t>
+  </si>
+  <si>
     <t>HU-013</t>
   </si>
   <si>
@@ -366,6 +420,15 @@
     <t>El profesional se asocia a una institución y a servicios válidos. • No se crean asociaciones duplicadas equivalentes. • Los cambios relevantes quedan auditados.</t>
   </si>
   <si>
+    <t>feat/professional-administration</t>
+  </si>
+  <si>
+    <t>HU-013 · Done</t>
+  </si>
+  <si>
+    <t>Administración de profesionales y asociaciones implementada.</t>
+  </si>
+  <si>
     <t>HU-014</t>
   </si>
   <si>
@@ -384,6 +447,15 @@
     <t>No se aceptan rangos inválidos o superpuestos cuando generen conflicto. • Los bloqueos impiden nuevas reservas en el periodo afectado. • La agenda refleja los cambios de disponibilidad.</t>
   </si>
   <si>
+    <t>feat/availability-administration</t>
+  </si>
+  <si>
+    <t>HU-014 · Done</t>
+  </si>
+  <si>
+    <t>Disponibilidad, materialización de cupos y bloqueos implementados.</t>
+  </si>
+  <si>
     <t>HU-015</t>
   </si>
   <si>
@@ -399,6 +471,15 @@
     <t>La agenda puede filtrarse por los criterios definidos. • Cada cita muestra estado y datos operativos relevantes. • El usuario sólo consulta sedes/recursos dentro de su ámbito autorizado.</t>
   </si>
   <si>
+    <t>feat/institutional-agenda</t>
+  </si>
+  <si>
+    <t>HU-015 · Done</t>
+  </si>
+  <si>
+    <t>Agenda institucional con filtros y trazabilidad de estados implementada.</t>
+  </si>
+  <si>
     <t>HU-016</t>
   </si>
   <si>
@@ -417,6 +498,15 @@
     <t>El flujo muestra al menos cupo, candidatos, oferta y estado actual. • La vista distingue operación automática de intervención manual autorizada. • Cada paso crítico posee trazabilidad.</t>
   </si>
   <si>
+    <t>feat/reassignment-supervision</t>
+  </si>
+  <si>
+    <t>HU-016 · Done</t>
+  </si>
+  <si>
+    <t>Consulta read-only de reasignación con trazabilidad y política implementada.</t>
+  </si>
+  <si>
     <t>HU-017</t>
   </si>
   <si>
@@ -441,6 +531,15 @@
     <t>Sólo roles autorizados registran asistencia/inasistencia. • No se registra asistencia sobre una cita cancelada. • El cambio queda persistido y auditado.</t>
   </si>
   <si>
+    <t>feat/appointment-attendance</t>
+  </si>
+  <si>
+    <t>HU-017 · Done</t>
+  </si>
+  <si>
+    <t>Registro de ATENDIDA/INASISTENCIA implementado con control de transiciones.</t>
+  </si>
+  <si>
     <t>HU-018</t>
   </si>
   <si>
@@ -456,6 +555,15 @@
     <t>Sólo administradores autorizados pueden cambiar parámetros. • Los valores deben respetar límites definidos por el sistema. • Los cambios quedan versionados o auditados y no alteran retroactivamente decisiones cerradas.</t>
   </si>
   <si>
+    <t>feat/reassignment-policy</t>
+  </si>
+  <si>
+    <t>HU-018 · Done</t>
+  </si>
+  <si>
+    <t>Políticas versionadas e inmutables de reasignación implementadas.</t>
+  </si>
+  <si>
     <t>HU-019</t>
   </si>
   <si>
@@ -477,6 +585,15 @@
     <t>Los indicadores se calculan a partir de datos persistidos. • Los filtros respetan el ámbito institucional. • Los resultados distinguen cancelaciones, ofertas, aceptaciones, expiraciones y cupos recuperados cuando corresponda.</t>
   </si>
   <si>
+    <t>feat/reports-indicators · PR #84</t>
+  </si>
+  <si>
+    <t>HU-019 · Done</t>
+  </si>
+  <si>
+    <t>Indicadores institucionales implementados y validados.</t>
+  </si>
+  <si>
     <t>HU-020</t>
   </si>
   <si>
@@ -495,297 +612,171 @@
     <t>El auditor posee acceso de lectura sin capacidad de alterar eventos. • La bitácora permite identificar actor/sistema, fecha, acción y recurso afectado según corresponda. • Los logs no exponen secretos o credenciales.</t>
   </si>
   <si>
+    <t>feat/audit-trail · PR #86</t>
+  </si>
+  <si>
+    <t>HU-020 · Done</t>
+  </si>
+  <si>
+    <t>Auditoría read-only e instrumentación de eventos relevantes implementadas y validadas.</t>
+  </si>
+  <si>
+    <t>HU-021</t>
+  </si>
+  <si>
+    <t>Como usuario de CitaJusta, quiero gestionar desde la Web mi participación en listas de espera y sus preferencias, para inscribirme, ajustar mis condiciones de atención y retirarme cuando corresponda.</t>
+  </si>
+  <si>
+    <t>Gestionar lista de espera y preferencias desde la Web</t>
+  </si>
+  <si>
+    <t>Por estimar</t>
+  </si>
+  <si>
+    <t>HU-007 / HU-008 Web</t>
+  </si>
+  <si>
+    <t>El usuario autenticado puede consultar e ingresar a listas válidas. • Puede configurar días, rangos y sedes preferidas. • Puede retirarse. • La UI usa respuestas reales y no replica ranking/elegibilidad.</t>
+  </si>
+  <si>
+    <t>feat/web-waitlist · PR #89 · merge c291d17</t>
+  </si>
+  <si>
+    <t>HU-021 · Done</t>
+  </si>
+  <si>
+    <t>Validación real Web + API + PostgreSQL: alta ACTIVE, preferencias persistentes y retiro. Web 56/56; development/seed 11/11; Waitlist E2E 24/24.</t>
+  </si>
+  <si>
+    <t>HU-022</t>
+  </si>
+  <si>
+    <t>Como usuario de CitaJusta, quiero visualizar y responder desde la Web las ofertas de reasignación que reciba, para aceptar una nueva hora compatible o rechazarla de forma segura.</t>
+  </si>
+  <si>
+    <t>Gestionar ofertas de reasignación desde la Web</t>
+  </si>
+  <si>
+    <t>HU-009 / HU-010 / HU-011 Web</t>
+  </si>
+  <si>
+    <t>La Web muestra ofertas reales y su expiresAt. • Permite aceptar/rechazar mediante los endpoints reales. • La aceptación transfiere la cita existente. • El rechazo no crea una cita. • El cliente no recalcula elegibilidad ni ranking.</t>
+  </si>
+  <si>
+    <t>feat/web-reassignment-offers · PR #93 · merge 5701ab7</t>
+  </si>
+  <si>
+    <t>HU-022 · Done</t>
+  </si>
+  <si>
+    <t>Validación completa Web + API + PostgreSQL: ACCEPT transfirió cita AGENDADA; REJECT no creó cita; oferta vencida deshabilitada sin mutación desde el cliente.</t>
+  </si>
+  <si>
+    <t>HU-023</t>
+  </si>
+  <si>
+    <t>Ofertas / Reasignación</t>
+  </si>
+  <si>
+    <t>Como sistema CitaJusta, quiero expirar automáticamente las ofertas vencidas y continuar con el siguiente candidato elegible, para recuperar cupos liberados sin depender de intervención manual.</t>
+  </si>
+  <si>
+    <t>Automatizar expiración y continuidad de reasignación</t>
+  </si>
+  <si>
+    <t>RF-029 / RF-030 / RF-036</t>
+  </si>
+  <si>
+    <t>Una oferta PENDING vencida pasa de forma persistente a EXPIRED. • La continuidad genera como máximo una siguiente oferta. • Sin candidatos el proceso queda EXHAUSTED. • Cupo/contexto inutilizable cierra CANCELLED. • La operación es idempotente, transaccional y segura ante concurrencia.</t>
+  </si>
+  <si>
+    <t>feat/automatic-offer-expiration · PR #96 · merge 109b1c9</t>
+  </si>
+  <si>
+    <t>HU-023 · Done</t>
+  </si>
+  <si>
+    <t>Runner interno sin dependencias nuevas. Auditoría OFFER_EXPIRED. Validación: API 368/368; E2E expiración 10/10; reasignaciones 20/20; audit 11/11; policy 13/13; reports 15/15; checkpoint 1/1.</t>
+  </si>
+  <si>
+    <t>HU-024</t>
+  </si>
+  <si>
+    <t>Notificaciones</t>
+  </si>
+  <si>
+    <t>Como usuario de CitaJusta, quiero recibir y consultar notificaciones internas sobre eventos importantes de mis citas, lista de espera y ofertas, para mantenerme informado sin depender de servicios externos.</t>
+  </si>
+  <si>
+    <t>Implementar notificaciones internas</t>
+  </si>
+  <si>
+    <t>RF-034</t>
+  </si>
+  <si>
+    <t>Las notificaciones se persisten dentro de las transacciones reales del dominio. • Sólo el destinatario autenticado puede consultarlas o marcarlas como leídas. • Reintentos idempotentes no generan duplicados. • La Web muestra contador, listado y lectura persistente.</t>
+  </si>
+  <si>
+    <t>feat/internal-notifications · PR #99 · merge b1bff30</t>
+  </si>
+  <si>
+    <t>HU-024 · Done</t>
+  </si>
+  <si>
+    <t>Ocho eventos integrados. API /notifications/me + unread-count + read. Web /notificaciones. Validación: nuevos API 6/6; E2E notifications 8/8; API dirigida 157/157; regresión crítica 87/87; Web 83/83; prueba manual de lectura y logout/login PASS.</t>
+  </si>
+  <si>
+    <t>HU-025</t>
+  </si>
+  <si>
+    <t>Como sistema CitaJusta, quiero iniciar automáticamente la reasignación cuando una cancelación libera un cupo reutilizable, para ofrecerlo a candidatos compatibles sin intervención administrativa.</t>
+  </si>
+  <si>
+    <t>Iniciar reasignación automática tras cancelación</t>
+  </si>
+  <si>
+    <t>Refuerzo RF-022 a RF-030</t>
+  </si>
+  <si>
+    <t>Una cancelación que libera un cupo reutilizable inicia la reasignación en la misma transacción. • No crea procesos/ofertas duplicados. • Sin candidatos elegibles queda EXHAUSTED. • Cupos no reutilizables permiten completar la cancelación sin procesos parciales.</t>
+  </si>
+  <si>
+    <t>feat/automatic-reassignment-start · PR #105 · merge ea33e9f</t>
+  </si>
+  <si>
+    <t>CitaJusta #103 · Done</t>
+  </si>
+  <si>
+    <t>Validación: API 390/390; E2E automatic-start 8/8; build y regresión relacionada PASS. Inicio automático auditado como SYSTEM y cancelación como USER.</t>
+  </si>
+  <si>
+    <t>HU-026</t>
+  </si>
+  <si>
+    <t>Como usuario de CitaJusta, quiero elegir una fecha específica o una búsqueda flexible, para encontrar disponibilidad de acuerdo con el día en que necesito atenderme.</t>
+  </si>
+  <si>
+    <t>Buscar disponibilidad por fecha específica</t>
+  </si>
+  <si>
+    <t>Permite Fecha específica mediante calendario o modo flexible 7/14/30 días. • Rechaza fechas pasadas. • Hoy inicia desde la hora actual. • Respeta calendario local y cambios DST. • Mantiene el mismo contrato from/to del backend.</t>
+  </si>
+  <si>
+    <t>feat/availability-date-search · PR #107 · merge ec427a4</t>
+  </si>
+  <si>
+    <t>HU-026 · Done</t>
+  </si>
+  <si>
+    <t>Validación: fechas 10/10; UI 16/16; Web 95/95; typecheck/build PASS. Prueba manual: 4 cupos reales coincidentes entre búsqueda flexible y fecha específica.</t>
+  </si>
+  <si>
     <t>Indicador</t>
   </si>
   <si>
     <t>Valor</t>
   </si>
   <si>
-    <t>Versión 1.7 · Actualización 22-09-2026 · Backend HU-001 a HU-020 completado · HU-021 a HU-026 Done · MVP Web cerrado.</t>
-  </si>
-  <si>
-    <t>feat/waitlist-entry</t>
-  </si>
-  <si>
-    <t>HU-007 · Done</t>
-  </si>
-  <si>
-    <t>Alta y consulta de lista de espera implementadas y validadas contra PostgreSQL real.</t>
-  </si>
-  <si>
-    <t>feat/waitlist-preferences</t>
-  </si>
-  <si>
-    <t>HU-008 · Done</t>
-  </si>
-  <si>
-    <t>Preferencias y retiro implementados; E2E HU-007/HU-008 real 24/24 PASS.</t>
-  </si>
-  <si>
-    <t>feat/reassignment-offers</t>
-  </si>
-  <si>
-    <t>HU-009 · Done</t>
-  </si>
-  <si>
-    <t>Generación de oferta, ranking/snapshot y TTL implementados en backend.</t>
-  </si>
-  <si>
-    <t>feat/accept-reassignment-offer</t>
-  </si>
-  <si>
-    <t>HU-010 · Done</t>
-  </si>
-  <si>
-    <t>Aceptación transaccional e idempotente implementada con transferencia segura de la cita.</t>
-  </si>
-  <si>
-    <t>feat/reject-reassignment-offer</t>
-  </si>
-  <si>
-    <t>HU-011 · Done</t>
-  </si>
-  <si>
-    <t>Rechazo y continuidad/exhaustión del flujo implementados.</t>
-  </si>
-  <si>
-    <t>feat/catalog-administration</t>
-  </si>
-  <si>
-    <t>HU-012 · Done</t>
-  </si>
-  <si>
-    <t>Administración de sedes/servicios implementada con permisos y activación/desactivación.</t>
-  </si>
-  <si>
-    <t>feat/professional-administration</t>
-  </si>
-  <si>
-    <t>HU-013 · Done</t>
-  </si>
-  <si>
-    <t>Administración de profesionales y asociaciones implementada.</t>
-  </si>
-  <si>
-    <t>feat/availability-administration</t>
-  </si>
-  <si>
-    <t>HU-014 · Done</t>
-  </si>
-  <si>
-    <t>Disponibilidad, materialización de cupos y bloqueos implementados.</t>
-  </si>
-  <si>
-    <t>feat/institutional-agenda</t>
-  </si>
-  <si>
-    <t>HU-015 · Done</t>
-  </si>
-  <si>
-    <t>Agenda institucional con filtros y trazabilidad de estados implementada.</t>
-  </si>
-  <si>
-    <t>feat/reassignment-supervision</t>
-  </si>
-  <si>
-    <t>HU-016 · Done</t>
-  </si>
-  <si>
-    <t>Consulta read-only de reasignación con trazabilidad y política implementada.</t>
-  </si>
-  <si>
-    <t>feat/appointment-attendance</t>
-  </si>
-  <si>
-    <t>HU-017 · Done</t>
-  </si>
-  <si>
-    <t>Registro de ATENDIDA/INASISTENCIA implementado con control de transiciones.</t>
-  </si>
-  <si>
-    <t>feat/reassignment-policy</t>
-  </si>
-  <si>
-    <t>HU-018 · Done</t>
-  </si>
-  <si>
-    <t>Políticas versionadas e inmutables de reasignación implementadas.</t>
-  </si>
-  <si>
-    <t>feat/reports-indicators · PR #84</t>
-  </si>
-  <si>
-    <t>HU-019 · Done</t>
-  </si>
-  <si>
-    <t>Indicadores institucionales implementados y validados.</t>
-  </si>
-  <si>
-    <t>feat/audit-trail · PR #86</t>
-  </si>
-  <si>
-    <t>HU-020 · Done</t>
-  </si>
-  <si>
-    <t>Auditoría read-only e instrumentación de eventos relevantes implementadas y validadas.</t>
-  </si>
-  <si>
-    <t>HU-021</t>
-  </si>
-  <si>
-    <t>Como usuario de CitaJusta, quiero gestionar desde la Web mi participación en listas de espera y sus preferencias, para inscribirme, ajustar mis condiciones de atención y retirarme cuando corresponda.</t>
-  </si>
-  <si>
-    <t>Gestionar lista de espera y preferencias desde la Web</t>
-  </si>
-  <si>
-    <t>Por estimar</t>
-  </si>
-  <si>
-    <t>HU-007 / HU-008 Web</t>
-  </si>
-  <si>
-    <t>El usuario autenticado puede consultar e ingresar a listas válidas. • Puede configurar días, rangos y sedes preferidas. • Puede retirarse. • La UI usa respuestas reales y no replica ranking/elegibilidad.</t>
-  </si>
-  <si>
-    <t>feat/web-waitlist · PR #89 · merge c291d17</t>
-  </si>
-  <si>
-    <t>HU-021 · Done</t>
-  </si>
-  <si>
-    <t>Validación real Web + API + PostgreSQL: alta ACTIVE, preferencias persistentes y retiro. Web 56/56; development/seed 11/11; Waitlist E2E 24/24.</t>
-  </si>
-  <si>
-    <t>HU-022</t>
-  </si>
-  <si>
-    <t>Como usuario de CitaJusta, quiero visualizar y responder desde la Web las ofertas de reasignación que reciba, para aceptar una nueva hora compatible o rechazarla de forma segura.</t>
-  </si>
-  <si>
-    <t>Gestionar ofertas de reasignación desde la Web</t>
-  </si>
-  <si>
-    <t>HU-009 / HU-010 / HU-011 Web</t>
-  </si>
-  <si>
-    <t>La Web muestra ofertas reales y su expiresAt. • Permite aceptar/rechazar mediante los endpoints reales. • La aceptación transfiere la cita existente. • El rechazo no crea una cita. • El cliente no recalcula elegibilidad ni ranking.</t>
-  </si>
-  <si>
-    <t>feat/web-reassignment-offers · PR #93 · merge 5701ab7</t>
-  </si>
-  <si>
-    <t>HU-022 · Done</t>
-  </si>
-  <si>
-    <t>Validación completa Web + API + PostgreSQL: ACCEPT transfirió cita AGENDADA; REJECT no creó cita; oferta vencida deshabilitada sin mutación desde el cliente.</t>
-  </si>
-  <si>
-    <t>HU-023</t>
-  </si>
-  <si>
-    <t>Ofertas / Reasignación</t>
-  </si>
-  <si>
-    <t>Como sistema CitaJusta, quiero expirar automáticamente las ofertas vencidas y continuar con el siguiente candidato elegible, para recuperar cupos liberados sin depender de intervención manual.</t>
-  </si>
-  <si>
-    <t>Automatizar expiración y continuidad de reasignación</t>
-  </si>
-  <si>
-    <t>RF-029 / RF-030 / RF-036</t>
-  </si>
-  <si>
-    <t>Una oferta PENDING vencida pasa de forma persistente a EXPIRED. • La continuidad genera como máximo una siguiente oferta. • Sin candidatos el proceso queda EXHAUSTED. • Cupo/contexto inutilizable cierra CANCELLED. • La operación es idempotente, transaccional y segura ante concurrencia.</t>
-  </si>
-  <si>
-    <t>feat/automatic-offer-expiration · PR #96 · merge 109b1c9</t>
-  </si>
-  <si>
-    <t>HU-023 · Done</t>
-  </si>
-  <si>
-    <t>Runner interno sin dependencias nuevas. Auditoría OFFER_EXPIRED. Validación: API 368/368; E2E expiración 10/10; reasignaciones 20/20; audit 11/11; policy 13/13; reports 15/15; checkpoint 1/1.</t>
-  </si>
-  <si>
-    <t>HU-024</t>
-  </si>
-  <si>
-    <t>Notificaciones</t>
-  </si>
-  <si>
-    <t>Como usuario de CitaJusta, quiero recibir y consultar notificaciones internas sobre eventos importantes de mis citas, lista de espera y ofertas, para mantenerme informado sin depender de servicios externos.</t>
-  </si>
-  <si>
-    <t>Implementar notificaciones internas</t>
-  </si>
-  <si>
-    <t>RF-034</t>
-  </si>
-  <si>
-    <t>Las notificaciones se persisten dentro de las transacciones reales del dominio. • Sólo el destinatario autenticado puede consultarlas o marcarlas como leídas. • Reintentos idempotentes no generan duplicados. • La Web muestra contador, listado y lectura persistente.</t>
-  </si>
-  <si>
-    <t>feat/internal-notifications · PR #99 · merge b1bff30</t>
-  </si>
-  <si>
-    <t>HU-024 · Done</t>
-  </si>
-  <si>
-    <t>Ocho eventos integrados. API /notifications/me + unread-count + read. Web /notificaciones. Validación: nuevos API 6/6; E2E notifications 8/8; API dirigida 157/157; regresión crítica 87/87; Web 83/83; prueba manual de lectura y logout/login PASS.</t>
-  </si>
-  <si>
-    <t>HU-025</t>
-  </si>
-  <si>
-    <t>Como sistema CitaJusta, quiero iniciar automáticamente la reasignación cuando una cancelación libera un cupo reutilizable, para ofrecerlo a candidatos compatibles sin intervención administrativa.</t>
-  </si>
-  <si>
-    <t>Iniciar reasignación automática tras cancelación</t>
-  </si>
-  <si>
-    <t>Refuerzo RF-022 a RF-030</t>
-  </si>
-  <si>
-    <t>Una cancelación que libera un cupo reutilizable inicia la reasignación en la misma transacción. • No crea procesos/ofertas duplicados. • Sin candidatos elegibles queda EXHAUSTED. • Cupos no reutilizables permiten completar la cancelación sin procesos parciales.</t>
-  </si>
-  <si>
-    <t>feat/automatic-reassignment-start · PR #105 · merge ea33e9f</t>
-  </si>
-  <si>
-    <t>CitaJusta #103 · Done</t>
-  </si>
-  <si>
-    <t>Validación: API 390/390; E2E automatic-start 8/8; build y regresión relacionada PASS. Inicio automático auditado como SYSTEM y cancelación como USER.</t>
-  </si>
-  <si>
-    <t>HU-026</t>
-  </si>
-  <si>
-    <t>Como usuario de CitaJusta, quiero elegir una fecha específica o una búsqueda flexible, para encontrar disponibilidad de acuerdo con el día en que necesito atenderme.</t>
-  </si>
-  <si>
-    <t>Buscar disponibilidad por fecha específica</t>
-  </si>
-  <si>
-    <t>Permite Fecha específica mediante calendario o modo flexible 7/14/30 días. • Rechaza fechas pasadas. • Hoy inicia desde la hora actual. • Respeta calendario local y cambios DST. • Mantiene el mismo contrato from/to del backend.</t>
-  </si>
-  <si>
-    <t>feat/availability-date-search · PR #107 · merge ec427a4</t>
-  </si>
-  <si>
-    <t>HU-026 · Done</t>
-  </si>
-  <si>
-    <t>Validación: fechas 10/10; UI 16/16; Web 95/95; typecheck/build PASS. Prueba manual: 4 cupos reales coincidentes entre búsqueda flexible y fecha específica.</t>
-  </si>
-  <si>
-    <t>Nota: HU-001 a HU-020 mantienen sus Story Points históricos (105 SP). HU-021 a HU-026 permanecen Por estimar hasta refinamiento formal del Scrum Team.</t>
-  </si>
-  <si>
-    <t>CITAJUSTA — RESUMEN DEL PRODUCT BACKLOG (ACTUALIZADO 22-09-2026)</t>
-  </si>
-  <si>
     <t>Historias</t>
   </si>
   <si>
@@ -819,18 +810,102 @@
     <t>Notas de actualización</t>
   </si>
   <si>
+    <t>Último avance técnico incorporado al Backlog</t>
+  </si>
+  <si>
+    <t>Versión 1.8 · Actualización 23-09-2026 · HU-001 a HU-029 Done · MVP Web cerrado · Sprint 7 Desktop/Tauri en progreso.</t>
+  </si>
+  <si>
+    <t>HU-027</t>
+  </si>
+  <si>
+    <t>Desktop institucional</t>
+  </si>
+  <si>
+    <t>Inicializar la aplicación institucional de escritorio con Tauri + React + TypeScript para disponer de una base nativa que consuma la misma API REST de CitaJusta.</t>
+  </si>
+  <si>
+    <t>Inicializar aplicación Desktop institucional con Tauri</t>
+  </si>
+  <si>
+    <t>Fundación Desktop / interfaz institucional</t>
+  </si>
+  <si>
+    <t>Existe apps/desktop dentro del monorepo. • Tauri 2 + React/Vite/TypeScript compila y abre correctamente. • La shell institucional queda preparada sin duplicar reglas de negocio en Rust/Tauri.</t>
+  </si>
+  <si>
+    <t>feat/desktop-tauri-foundation · commit 01ff1b1 · PR #112 · merge 6adab82</t>
+  </si>
+  <si>
+    <t>HU-027 · Done</t>
+  </si>
+  <si>
+    <t>Fundación Desktop creada y validada con build frontend, cargo check y ejecución nativa Tauri.</t>
+  </si>
+  <si>
+    <t>HU-028</t>
+  </si>
+  <si>
+    <t>Como usuario institucional, quiero iniciar sesión de forma segura en CitaJusta Desktop, para acceder a la API con mi contexto autorizado sin persistir tokens de forma insegura.</t>
+  </si>
+  <si>
+    <t>Autenticación Desktop y client-core compartido</t>
+  </si>
+  <si>
+    <t>Auth Desktop / cliente compartido</t>
+  </si>
+  <si>
+    <t>Login real contra API. • Perfil/contexto provienen del backend. • Tokens permanecen sólo en memoria. • Web y Desktop comparten HTTP/sesión mediante @citajusta/client-core. • Logout elimina la sesión local.</t>
+  </si>
+  <si>
+    <t>feat/desktop-auth-api · commit 46fb85f · PR #113 · merge ae151b3</t>
+  </si>
+  <si>
+    <t>HU-028 · Done</t>
+  </si>
+  <si>
+    <t>Validación: Web 95/95; Desktop 7/7; client-core 2/2; builds y cargo check PASS; login/logout manual en Tauri PASS.</t>
+  </si>
+  <si>
+    <t>HU-029</t>
+  </si>
+  <si>
+    <t>Como usuario institucional autorizado, quiero gestionar las sedes y servicios de mi institución desde CitaJusta Desktop, para mantener actualizado el catálogo institucional utilizado por agenda, profesionales, disponibilidad y procesos de atención.</t>
+  </si>
+  <si>
+    <t>Gestionar sedes y servicios desde Desktop</t>
+  </si>
+  <si>
+    <t>HU-012 Desktop / RBAC administrativo</t>
+  </si>
+  <si>
+    <t>Lecturas administrativas respetan tenant y scope. • Crear/editar/activar/inactivar sedes y servicios usa permisos explícitos. • Servicios administran branchIds y categorías reales. • GET públicos existentes conservan su contrato.</t>
+  </si>
+  <si>
+    <t>feat/desktop-branch-service-management · commit f58c742 · merge e1cdb2e</t>
+  </si>
+  <si>
+    <t>HU-029 · Done</t>
+  </si>
+  <si>
+    <t>Validación: API 394/394; backend enfocado 34/34; E2E catálogo 15/15; Web 95/95; Desktop 16/16; client-core 4/4; Prisma/build/cargo/diff PASS y prueba manual Tauri/PostgreSQL completa.</t>
+  </si>
+  <si>
+    <t>Nota: HU-001 a HU-020 mantienen sus Story Points históricos (105 SP). HU-021 a HU-029 permanecen Por estimar hasta refinamiento formal del Scrum Team. HU-027 a HU-029 documentan el inicio de Sprint 7 Desktop/Tauri y no alteran retrospectivamente Sprints cerrados.</t>
+  </si>
+  <si>
+    <t>CITAJUSTA — RESUMEN DEL PRODUCT BACKLOG (ACTUALIZADO 23-09-2026)</t>
+  </si>
+  <si>
     <t>• Backend HU-001 a HU-020 Done.
-• HU-021/022 Web Done (PR #89/#93).
-• HU-023/024 expiración + notificaciones Done (PR #96/#99).
-• HU-025 inicio automático tras cancelación Done (PR #105).
-• HU-026 fecha específica/flexible Done (PR #107).
-• MVP Web cerrado; HU-021 a HU-026 mantienen Story Points Por estimar.</t>
-  </si>
-  <si>
-    <t>Último avance técnico incorporado al Backlog</t>
-  </si>
-  <si>
-    <t>HU-025 y HU-026 completaron el cierre funcional del MVP Web: la cancelación dispara automáticamente la reasignación cuando corresponde y el buscador permite fecha específica o rango flexible. Próximo foco: Desktop/Tauri institucional.</t>
+• HU-021 a HU-026 cerraron el MVP Web.
+• HU-027 fundó apps/desktop con Tauri 2.
+• HU-028 incorporó autenticación Desktop y @citajusta/client-core.
+• HU-029 incorporó gestión institucional real de sedes y servicios.
+• HU-021 a HU-029 mantienen Story Points Por estimar.</t>
+  </si>
+  <si>
+    <t>Sprint 7 Desktop/Tauri en progreso. HU-027 (PR #112, merge 6adab82), HU-028 (PR #113, merge ae151b3) y HU-029 (commit f58c742, merge e1cdb2e) están Done. El siguiente PBI Desktop queda pendiente de refinamiento antes de incorporarlo al backlog.</t>
   </si>
 </sst>
 </file>
@@ -899,11 +974,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7F9FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFB6D7A8"/>
       </patternFill>
     </fill>
@@ -919,8 +989,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79995117038483843"/>
+        <fgColor theme="9" tint="0.79992065187536243"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -930,7 +1006,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -1137,22 +1213,102 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1167,23 +1323,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1201,7 +1366,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1209,25 +1374,46 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1334,7 +1520,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>26</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1375,7 +1561,7 @@
               </c15:filteredCategoryTitle>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2A6C-41C8-8427-52B2FF6E7483}"/>
+              <c16:uniqueId val="{00000000-151B-4442-A64E-99C17721FD3B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1803,40 +1989,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="27.75" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+      <c r="A2" s="44" t="s">
+        <v>259</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
     </row>
     <row r="4" spans="1:14" ht="33.75" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -2181,27 +2367,27 @@
         <v>76</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>156</v>
+        <v>77</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>157</v>
+        <v>78</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>158</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="43.5" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>19</v>
@@ -2216,36 +2402,36 @@
         <v>21</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>159</v>
+        <v>85</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>160</v>
+        <v>86</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>161</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="43.5" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>19</v>
@@ -2254,42 +2440,42 @@
         <v>8</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>162</v>
+        <v>95</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>163</v>
+        <v>96</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>164</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="43.5" customHeight="1">
       <c r="A14" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="C14" s="1" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>19</v>
@@ -2298,42 +2484,42 @@
         <v>8</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>165</v>
+        <v>103</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="43.5" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>19</v>
@@ -2342,42 +2528,42 @@
         <v>3</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>21</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>168</v>
+        <v>111</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>169</v>
+        <v>112</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>170</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="43.5" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>19</v>
@@ -2392,36 +2578,36 @@
         <v>21</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>171</v>
+        <v>120</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>172</v>
+        <v>121</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>173</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="43.5" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>19</v>
@@ -2436,36 +2622,36 @@
         <v>21</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>174</v>
+        <v>128</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>176</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="43.5" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>19</v>
@@ -2480,36 +2666,36 @@
         <v>31</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>177</v>
+        <v>137</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>178</v>
+        <v>138</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>179</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="43.5" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>19</v>
@@ -2524,36 +2710,36 @@
         <v>21</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>180</v>
+        <v>145</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>181</v>
+        <v>146</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="43.5" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>121</v>
+        <v>148</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>19</v>
@@ -2562,42 +2748,42 @@
         <v>8</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>125</v>
+        <v>152</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>23</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>183</v>
+        <v>154</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>184</v>
+        <v>155</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="43.5" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>129</v>
+        <v>159</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>19</v>
@@ -2609,39 +2795,39 @@
         <v>49</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>133</v>
+        <v>163</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>134</v>
+        <v>164</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>187</v>
+        <v>166</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>188</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="43.5" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>136</v>
+        <v>169</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>137</v>
+        <v>170</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>19</v>
@@ -2650,42 +2836,42 @@
         <v>8</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>21</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>133</v>
+        <v>163</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>139</v>
+        <v>172</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="43.5" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>140</v>
+        <v>176</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>141</v>
+        <v>177</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>142</v>
+        <v>178</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>143</v>
+        <v>179</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>19</v>
@@ -2694,92 +2880,92 @@
         <v>5</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>144</v>
+        <v>180</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>145</v>
+        <v>181</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>133</v>
+        <v>163</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="L23" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="43.5" customHeight="1">
+      <c r="A24" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="12">
+        <v>5</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="L24" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="M23" s="1" t="s">
+      <c r="M24" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="N23" s="1" t="s">
+      <c r="N24" s="12" t="s">
         <v>194</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="43.5" customHeight="1">
-      <c r="A24" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="B24" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="C24" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D24" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="30">
-        <v>5</v>
-      </c>
-      <c r="G24" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="H24" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="I24" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="J24" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="K24" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="L24" s="30" t="s">
-        <v>195</v>
-      </c>
-      <c r="M24" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="N24" s="30" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="67.5" customHeight="1">
       <c r="A25" s="10" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>72</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="E25" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="E25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="G25" s="10" t="s">
         <v>49</v>
@@ -2788,221 +2974,221 @@
         <v>21</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="J25" s="10" t="s">
         <v>23</v>
       </c>
       <c r="K25" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="L25" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="M25" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="N25" s="10" t="s">
         <v>203</v>
-      </c>
-      <c r="L25" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="M25" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="N25" s="10" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="70.5" customHeight="1">
       <c r="A26" s="10" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="E26" s="30" t="s">
+        <v>206</v>
+      </c>
+      <c r="E26" s="12" t="s">
         <v>19</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H26" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="J26" s="10" t="s">
         <v>23</v>
       </c>
       <c r="K26" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="L26" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="M26" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="N26" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="L26" s="10" t="s">
+    </row>
+    <row r="27" spans="1:14" ht="69.95" customHeight="1">
+      <c r="A27" s="43" t="s">
         <v>212</v>
       </c>
-      <c r="M26" s="10" t="s">
+      <c r="B27" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="N26" s="10" t="s">
+      <c r="C27" s="13" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" ht="69.95" customHeight="1">
-      <c r="A27" s="31" t="s">
+      <c r="D27" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="E27" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H27" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="I27" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="J27" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K27" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="D27" s="32" t="s">
+      <c r="L27" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="E27" s="30" t="s">
+      <c r="M27" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="N27" s="13" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="69.95" customHeight="1">
+      <c r="A28" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="E28" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F27" s="32" t="s">
-        <v>201</v>
-      </c>
-      <c r="G27" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="H27" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="I27" s="32" t="s">
-        <v>219</v>
-      </c>
-      <c r="J27" s="32" t="s">
+      <c r="F28" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="J28" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="K27" s="32" t="s">
-        <v>220</v>
-      </c>
-      <c r="L27" s="32" t="s">
-        <v>221</v>
-      </c>
-      <c r="M27" s="32" t="s">
-        <v>222</v>
-      </c>
-      <c r="N27" s="32" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" ht="69.95" customHeight="1">
-      <c r="A28" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="B28" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C28" s="29" t="s">
+      <c r="K28" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="L28" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="E28" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="F28" s="29" t="s">
-        <v>201</v>
-      </c>
-      <c r="G28" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="H28" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="I28" s="29" t="s">
+      <c r="M28" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="J28" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="K28" s="29" t="s">
+      <c r="N28" s="11" t="s">
         <v>229</v>
-      </c>
-      <c r="L28" s="29" t="s">
-        <v>230</v>
-      </c>
-      <c r="M28" s="29" t="s">
-        <v>231</v>
-      </c>
-      <c r="N28" s="29" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="84.75" customHeight="1">
       <c r="A29" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="E29" s="30" t="s">
+        <v>232</v>
+      </c>
+      <c r="E29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>144</v>
+        <v>180</v>
       </c>
       <c r="H29" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J29" s="10" t="s">
         <v>23</v>
       </c>
       <c r="K29" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="L29" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="M29" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="N29" s="10" t="s">
         <v>237</v>
-      </c>
-      <c r="L29" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="M29" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="N29" s="10" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="87.75" customHeight="1">
       <c r="A30" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>37</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="E30" s="30" t="s">
+        <v>240</v>
+      </c>
+      <c r="E30" s="12" t="s">
         <v>19</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>144</v>
+        <v>180</v>
       </c>
       <c r="H30" s="10" t="s">
         <v>21</v>
@@ -3014,53 +3200,179 @@
         <v>23</v>
       </c>
       <c r="K30" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="L30" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="M30" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="N30" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="L30" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="M30" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="N30" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" ht="14.25" customHeight="1">
-      <c r="A31" s="33" t="s">
-        <v>248</v>
-      </c>
-      <c r="B31" s="33"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="33"/>
-      <c r="K31" s="33"/>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
-      <c r="N31" s="33"/>
-    </row>
-    <row r="32" spans="1:14" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1"/>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
+    </row>
+    <row r="31" spans="1:14" ht="69" customHeight="1">
+      <c r="A31" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="B31" s="32" t="s">
+        <v>261</v>
+      </c>
+      <c r="C31" s="32" t="s">
+        <v>262</v>
+      </c>
+      <c r="D31" s="32" t="s">
+        <v>263</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="G31" s="32" t="s">
+        <v>180</v>
+      </c>
+      <c r="H31" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="I31" s="32" t="s">
+        <v>264</v>
+      </c>
+      <c r="J31" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="K31" s="32" t="s">
+        <v>265</v>
+      </c>
+      <c r="L31" s="32" t="s">
+        <v>266</v>
+      </c>
+      <c r="M31" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="N31" s="32" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="63" customHeight="1">
+      <c r="A32" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="J32" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="K32" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="L32" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="M32" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="N32" s="10" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="55.5" customHeight="1">
+      <c r="A33" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="E33" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I33" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="J33" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="K33" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="L33" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="M33" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="N33" s="10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="22.5" customHeight="1"/>
+    <row r="35" spans="1:14" ht="15" customHeight="1"/>
+    <row r="36" spans="1:14" ht="15.75" hidden="1" customHeight="1"/>
+    <row r="37" spans="1:14" ht="15.75" hidden="1" customHeight="1"/>
+    <row r="38" spans="1:14" ht="15.75" hidden="1" customHeight="1"/>
+    <row r="39" spans="1:14" ht="15.75" hidden="1" customHeight="1"/>
+    <row r="40" spans="1:14" ht="15.75" customHeight="1"/>
+    <row r="41" spans="1:14" ht="15.75" customHeight="1"/>
+    <row r="42" spans="1:14" ht="18.75" customHeight="1"/>
+    <row r="43" spans="1:14" ht="15.75" customHeight="1">
+      <c r="B43" s="34" t="s">
+        <v>285</v>
+      </c>
+      <c r="C43" s="33"/>
+      <c r="D43" s="35"/>
+    </row>
+    <row r="44" spans="1:14" ht="15.75" customHeight="1">
+      <c r="B44" s="36"/>
+      <c r="C44" s="37"/>
+      <c r="D44" s="38"/>
+    </row>
+    <row r="45" spans="1:14" ht="15.75" customHeight="1">
+      <c r="B45" s="39"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="41"/>
+    </row>
+    <row r="46" spans="1:14" ht="15.75" customHeight="1"/>
+    <row r="47" spans="1:14" ht="15.75" customHeight="1"/>
+    <row r="48" spans="1:14" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
@@ -4017,9 +4329,9 @@
   <mergeCells count="3">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A31:N31"/>
+    <mergeCell ref="B43:D45"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E30">
+  <conditionalFormatting sqref="E5:E33">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>E5="Done"</formula>
     </cfRule>
@@ -4043,7 +4355,7 @@
     <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="G5:G24" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Sprint 3,Sprint 4,Sprint 5,Sprint 6,Sprint 7"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E5:E30" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" sqref="E5:E33" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Done,En progreso,Pendiente"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4068,37 +4380,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="57" customHeight="1">
-      <c r="A1" s="34" t="s">
-        <v>249</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="A1" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="30">
       <c r="A3" s="2" t="s">
-        <v>153</v>
+        <v>245</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>154</v>
+        <v>246</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B4" s="1">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="5" t="s">
@@ -4106,20 +4418,20 @@
       </c>
       <c r="E4" s="5">
         <f t="shared" ref="E4:E6" si="0">B6</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" ht="28.5">
       <c r="A5" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B5" s="1">
         <v>105</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="5" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E5" s="5">
         <f t="shared" si="0"/>
@@ -4127,16 +4439,16 @@
       </c>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:6" ht="28.5">
+    <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="1">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E6" s="5">
         <f t="shared" si="0"/>
@@ -4146,7 +4458,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B7" s="1">
         <v>0</v>
@@ -4158,7 +4470,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B8" s="5">
         <v>0</v>
@@ -4168,13 +4480,13 @@
         <v>7</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:6" ht="29.25">
       <c r="A9" s="5" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B9" s="5">
         <v>105</v>
@@ -4190,7 +4502,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="5" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B10" s="6">
         <v>1</v>
@@ -4206,7 +4518,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="5" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B11" s="5">
         <v>22</v>
@@ -4222,14 +4534,14 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="5" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B12" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="5" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E12" s="5">
         <v>8</v>
@@ -4241,10 +4553,10 @@
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="5" t="s">
-        <v>144</v>
+        <v>180</v>
       </c>
       <c r="E13" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F13" s="5"/>
     </row>
@@ -4253,18 +4565,18 @@
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E14" s="5">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F14" s="5"/>
     </row>
     <row r="15" spans="1:6" ht="15">
-      <c r="A15" s="15" t="s">
-        <v>260</v>
-      </c>
-      <c r="B15" s="16"/>
+      <c r="A15" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="B15" s="19"/>
       <c r="C15" s="3"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5" t="str">
@@ -4277,95 +4589,95 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="B16" s="18"/>
+      <c r="A16" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="B16" s="21"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="19"/>
-      <c r="B17" s="20"/>
+      <c r="A17" s="22"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="19"/>
-      <c r="B18" s="20"/>
+      <c r="A18" s="22"/>
+      <c r="B18" s="23"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="19"/>
-      <c r="B19" s="20"/>
+      <c r="A19" s="22"/>
+      <c r="B19" s="23"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="19"/>
-      <c r="B20" s="20"/>
+      <c r="A20" s="22"/>
+      <c r="B20" s="23"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
     </row>
     <row r="21" spans="1:6" ht="50.25" customHeight="1">
-      <c r="A21" s="21"/>
-      <c r="B21" s="22"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="25"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1"/>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="23" t="s">
-        <v>262</v>
-      </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="16"/>
+      <c r="A23" s="26" t="s">
+        <v>258</v>
+      </c>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="19"/>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A24" s="17" t="s">
-        <v>263</v>
-      </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="18"/>
+      <c r="A24" s="20" t="s">
+        <v>288</v>
+      </c>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="21"/>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A25" s="26"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="27"/>
+      <c r="A25" s="29"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="30"/>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A26" s="26"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="27"/>
+      <c r="A26" s="29"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="30"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A27" s="21"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="22"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="25"/>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1"/>
     <row r="29" spans="1:6" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
docs: fix product backlog note row
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Scrum/06_Product_Backlog_CitaJusta.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Scrum/06_Product_Backlog_CitaJusta.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Backlog" sheetId="1" r:id="R895418e10391461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R33ed29f45d0f4aa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Backlog" sheetId="1" r:id="R50655d6ff9bf4701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R221b4cf1e3274e74"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2061,7 +2061,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4e61acc413f4a60"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R256467bb80ae43ca"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4340,48 +4340,22 @@
       </x:c>
     </x:row>
     <x:row r="52" ht="34" customHeight="1">
-      <x:c r="A52" t="str">
-        <x:v>HU-040</x:v>
-      </x:c>
+      <x:c r="A52"/>
       <x:c r="B52" s="93" t="str">
         <x:v>Nota: HU-001 a HU-020 mantienen sus Story Points históricos (105 SP). HU-021 a HU-043 permanecen Por estimar hasta refinamiento/Planning formal. HU-030 a HU-038 documentan trabajo ya implementado en Sprint 7; HU-039 a HU-043 formalizan integraciones externas planificadas para Sprint 8 y no reescriben retrospectivamente Sprints cerrados.</x:v>
       </x:c>
-      <x:c r="C52" s="93" t="str">
-        <x:v>Como usuario, quiero iniciar sesión con mi cuenta Google, para acceder a CitaJusta mediante un método adicional de autenticación.</x:v>
-      </x:c>
-      <x:c r="D52" s="93" t="str">
-        <x:v>Integrar Google OAuth / OpenID Connect</x:v>
-      </x:c>
-      <x:c r="E52" s="93" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="F52" s="93" t="str">
-        <x:v>Por estimar</x:v>
-      </x:c>
-      <x:c r="G52" s="93" t="str">
-        <x:v>Sprint 8</x:v>
-      </x:c>
-      <x:c r="H52" s="93" t="str">
-        <x:v>Alta</x:v>
-      </x:c>
-      <x:c r="I52" s="93" t="str">
-        <x:v>RF-040</x:v>
-      </x:c>
-      <x:c r="J52" s="93" t="str">
-        <x:v>Objetivo</x:v>
-      </x:c>
-      <x:c r="K52" s="93" t="str">
-        <x:v>Google se incorpora como método adicional y no elimina el login actual. • La identidad OIDC se valida del lado servidor y se vincula de forma controlada a User. • Google no define roles/permisos institucionales. • Tokens y secretos del proveedor no se exponen al cliente ni a logs.</x:v>
-      </x:c>
-      <x:c r="L52" s="93" t="str">
-        <x:v>Planificada · Google OAuth/OIDC</x:v>
-      </x:c>
-      <x:c r="M52" s="93" t="str">
-        <x:v>Pendiente de crear/refinar</x:v>
-      </x:c>
-      <x:c r="N52" s="93" t="str">
-        <x:v>Debe preservar Auth, RBAC y AuthorizationContext existentes y definir una política segura de vinculación de cuentas.</x:v>
-      </x:c>
+      <x:c r="C52" s="93"/>
+      <x:c r="D52" s="93"/>
+      <x:c r="E52" s="93"/>
+      <x:c r="F52" s="93"/>
+      <x:c r="G52" s="93"/>
+      <x:c r="H52" s="93"/>
+      <x:c r="I52" s="93"/>
+      <x:c r="J52" s="93"/>
+      <x:c r="K52" s="93"/>
+      <x:c r="L52" s="93"/>
+      <x:c r="M52" s="93"/>
+      <x:c r="N52" s="93"/>
     </x:row>
     <x:row r="53" ht="15.75" customHeight="1"/>
     <x:row r="54" ht="15.75" customHeight="1"/>
@@ -5367,7 +5341,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc26970cf9694743"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec2d9d2d27d64d0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5586,9 +5560,8 @@
       <x:c r="D15" s="5" t="str">
         <x:v>Total</x:v>
       </x:c>
-      <x:c r="E15" s="5" t="n">
+      <x:c r="E15" s="5" t="str">
         <x:f t="shared" ref="E15:F15" si="1">""</x:f>
-        <x:v>43</x:v>
       </x:c>
       <x:c r="F15" s="5" t="str">
         <x:f t="shared" si="1"/>
@@ -6687,6 +6660,6 @@
     <x:mergeCell ref="A23:E25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa01985b34df4314"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc9bb9d212604568"/>
 </x:worksheet>
 </file>
</xml_diff>